<commit_message>
Doc (JDT) : UPDATE JDT
</commit_message>
<xml_diff>
--- a/jdt_chabal_damien.xlsx
+++ b/jdt_chabal_damien.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\347-docker-swarm-wordpress\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damie\Documents\GitHub\347-docker-swarm-wordpress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEAC245-C09D-41B1-848D-3B1E604ACCD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9177EBD2-A8A3-47A5-AED8-D8B9C071FE85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="4230" yWindow="1440" windowWidth="17250" windowHeight="14295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="55">
   <si>
     <t>Auteur:</t>
   </si>
@@ -152,6 +152,60 @@
   </si>
   <si>
     <t>Remplissage du JDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Étude de l'architecture Docker Swarm et des volumes partagés NFS                                       </t>
+  </si>
+  <si>
+    <t>Initialisation du cluster Swarm et jointure des 2 Workers</t>
+  </si>
+  <si>
+    <t>Installation et configuration du serveur NFS sur Worker</t>
+  </si>
+  <si>
+    <t>Rédaction des étapes 2 et 4 dans le README et mise à jour du jdt</t>
+  </si>
+  <si>
+    <t>Analyse des secrets Docker et séparation des réseaux</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Création des réseaux overlay front/back et de docker</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Configuration du service MariaDB avec contrainte de</t>
+  </si>
+  <si>
+    <t>Update jdt</t>
+  </si>
+  <si>
+    <t>Analyse de WordPress et partage NFS</t>
+  </si>
+  <si>
+    <t>Test de communication MariaDB - WordPress</t>
+  </si>
+  <si>
+    <t>Intégration du reverse proxy Nginx dans la stack Swarm</t>
+  </si>
+  <si>
+    <t>Validation de l'accès web HTTP et installation de wordpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentation de la configuration Nginx </t>
+  </si>
+  <si>
+    <t>Déploiement global de la stack via docker stack deploy</t>
+  </si>
+  <si>
+    <t>Test de répartition de charge sur les 3 réplique WordPress</t>
+  </si>
+  <si>
+    <t>Rédaction de l'étape Déploiement de la stack dans le readme</t>
+  </si>
+  <si>
+    <t>amélioration du projet</t>
+  </si>
+  <si>
+    <t>Rattrapage du test</t>
   </si>
 </sst>
 </file>
@@ -1159,19 +1213,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>45</c:v>
+                  <c:v>195</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>75</c:v>
+                  <c:v>460</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60</c:v>
+                  <c:v>275</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2014,16 +2068,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.25</c:v>
+                  <c:v>0.14772727272727273</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.41666666666666669</c:v>
+                  <c:v>0.34848484848484851</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.15909090909090909</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.33333333333333331</c:v>
+                  <c:v>0.20833333333333334</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4258,7 +4312,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 0 minutes</v>
+        <v>22 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4273,15 +4327,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>60</v>
+        <v>960</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>120</v>
+        <v>360</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>180</v>
+        <v>1320</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4452,15 +4506,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="62" t="str">
+      <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="30"/>
+        <v>36</v>
+      </c>
+      <c r="B12" s="30">
+        <v>46267</v>
+      </c>
       <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
+      <c r="D12" s="32">
+        <v>30</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
         <v>28</v>
@@ -4473,15 +4535,23 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
-      <c r="C13" s="35"/>
+        <v>36</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46267</v>
+      </c>
+      <c r="C13" s="35">
+        <v>1</v>
+      </c>
       <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="E13" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4491,15 +4561,23 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="62" t="str">
+      <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="31"/>
+        <v>36</v>
+      </c>
+      <c r="B14" s="30">
+        <v>46267</v>
+      </c>
+      <c r="C14" s="31">
+        <v>1</v>
+      </c>
       <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="E14" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>39</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -4509,15 +4587,23 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46274</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>20</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>40</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4527,183 +4613,301 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
+        <v>37</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46274</v>
+      </c>
+      <c r="C16" s="31">
+        <v>1</v>
+      </c>
       <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+      <c r="E16" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="str">
+      <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B17" s="34">
+        <v>46274</v>
+      </c>
       <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
+      <c r="D17" s="36">
+        <v>45</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G17" s="40"/>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+        <v>37</v>
+      </c>
+      <c r="B18" s="30">
+        <v>46274</v>
+      </c>
+      <c r="C18" s="31">
+        <v>1</v>
+      </c>
+      <c r="D18" s="32">
+        <v>20</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="str">
+      <c r="A19" s="63">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="34"/>
+        <v>38</v>
+      </c>
+      <c r="B19" s="34">
+        <v>46281</v>
+      </c>
       <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="D19" s="36">
+        <v>25</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="62" t="str">
+      <c r="A20" s="62">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
+        <v>38</v>
+      </c>
+      <c r="B20" s="30">
+        <v>46281</v>
+      </c>
+      <c r="C20" s="31">
+        <v>1</v>
+      </c>
       <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="E20" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>45</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="str">
+      <c r="A21" s="63">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="35"/>
+        <v>39</v>
+      </c>
+      <c r="B21" s="34">
+        <v>46288</v>
+      </c>
+      <c r="C21" s="35">
+        <v>1</v>
+      </c>
       <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="E21" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>46</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="62" t="str">
+      <c r="A22" s="62">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
+        <v>39</v>
+      </c>
+      <c r="B22" s="30">
+        <v>46288</v>
+      </c>
+      <c r="C22" s="31">
+        <v>1</v>
+      </c>
+      <c r="D22" s="32">
+        <v>20</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="str">
+      <c r="A23" s="63">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="34"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+        <v>40</v>
+      </c>
+      <c r="B23" s="34">
+        <v>46295</v>
+      </c>
+      <c r="C23" s="35">
+        <v>1</v>
+      </c>
+      <c r="D23" s="36">
+        <v>30</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="62" t="str">
+      <c r="A24" s="62">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B24" s="30">
+        <v>46295</v>
+      </c>
       <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="23"/>
+      <c r="D24" s="32">
+        <v>25</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>49</v>
+      </c>
       <c r="G24" s="39"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="str">
+      <c r="A25" s="63">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="34"/>
-      <c r="C25" s="35"/>
+        <v>40</v>
+      </c>
+      <c r="B25" s="34">
+        <v>46295</v>
+      </c>
+      <c r="C25" s="35">
+        <v>1</v>
+      </c>
       <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="23"/>
+      <c r="E25" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>50</v>
+      </c>
       <c r="G25" s="40"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="62" t="str">
+      <c r="A26" s="62">
         <f>IF(ISBLANK(B26),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="B26" s="30">
+        <v>46302</v>
+      </c>
+      <c r="C26" s="31">
+        <v>1</v>
+      </c>
       <c r="D26" s="32"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="23"/>
+      <c r="E26" s="33" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G26" s="39"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="63" t="str">
+      <c r="A27" s="63">
         <f>IF(ISBLANK(B27),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B27))</f>
-        <v/>
-      </c>
-      <c r="B27" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B27" s="34">
+        <v>46302</v>
+      </c>
       <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="23"/>
+      <c r="D27" s="36">
+        <v>25</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G27" s="40"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="62" t="str">
+      <c r="A28" s="62">
         <f>IF(ISBLANK(B28),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B28))</f>
-        <v/>
-      </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="31"/>
+        <v>41</v>
+      </c>
+      <c r="B28" s="30">
+        <v>46302</v>
+      </c>
+      <c r="C28" s="31">
+        <v>2</v>
+      </c>
       <c r="D28" s="32"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="22"/>
+      <c r="E28" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>53</v>
+      </c>
       <c r="G28" s="39"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="63" t="str">
+      <c r="A29" s="63">
         <f>IF(ISBLANK(B29),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B29))</f>
-        <v/>
-      </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="35"/>
+        <v>44</v>
+      </c>
+      <c r="B29" s="34">
+        <v>46323</v>
+      </c>
+      <c r="C29" s="35">
+        <v>3</v>
+      </c>
       <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
-      <c r="F29" s="22"/>
+      <c r="E29" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="G29" s="40"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -10876,15 +11080,15 @@
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>45</v>
+        <v>195</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10892,11 +11096,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 45 min</v>
+        <v>3 h 15 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.25</v>
+        <v>0.14772727272727273</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10913,15 +11117,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>360</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>75</v>
+        <v>460</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10929,11 +11133,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>1 h 15 min</v>
+        <v>7 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.41666666666666669</v>
+        <v>0.34848484848484851</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10950,15 +11154,15 @@
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="B8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="E8" s="76" t="str">
         <f>'Journal de travail'!M10</f>
@@ -10966,11 +11170,11 @@
       </c>
       <c r="F8" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>3 h 30 min</v>
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.15909090909090909</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -10987,15 +11191,15 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>155</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>60</v>
+        <v>275</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11003,11 +11207,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 00 min</v>
+        <v>4 h 35 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11024,7 +11228,7 @@
     <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E10,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E10,'Journal de travail'!$D$7:$D$532)</f>
@@ -11032,18 +11236,18 @@
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="E10" s="78" t="s">
         <v>28</v>
       </c>
       <c r="F10" s="79" t="str">
         <f t="shared" ref="F10" si="4">QUOTIENT(SUM(A10:B10),60)&amp;" h "&amp;TEXT(MOD(SUM(A10:B10),60), "00")&amp;" min"</f>
-        <v>0 h 00 min</v>
+        <v>3 h 00 min</v>
       </c>
       <c r="G10" s="80">
         <f>SUM(A10:B10)/$C$11</f>
-        <v>0</v>
+        <v>0.13636363636363635</v>
       </c>
       <c r="L10" s="69" t="s">
         <v>28</v>
@@ -11059,26 +11263,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>60</v>
+        <v>960</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>120</v>
+        <v>360</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>180</v>
+        <v>1320</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>18</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 00 min</v>
+        <v>22 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>3.3333333333333333E-2</v>
+        <v>0.24444444444444444</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>18</v>
@@ -11117,6 +11321,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="dfbaf9a740889adeb1cda0be194d08b7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4f25723b2930dbb90e2332f0c8c46e31" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -11317,27 +11541,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7F8341A-4C75-4689-8311-30F611A1EC8F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11354,25 +11579,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>